<commit_message>
Updated on 4 september
</commit_message>
<xml_diff>
--- a/12625732.xlsx
+++ b/12625732.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="77">
   <si>
     <t xml:space="preserve">My Data, My Code</t>
   </si>
@@ -243,6 +243,15 @@
   </si>
   <si>
     <t xml:space="preserve">weekend - no classes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">exam prep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">good progress on project</t>
+  </si>
+  <si>
+    <t xml:space="preserve">long lecture 10:20am-5pm, exhausted</t>
   </si>
 </sst>
 </file>
@@ -1659,114 +1668,234 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="18" t="str">
+      <c r="A18" s="13" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B18" s="14" t="n">
+        <v>445</v>
+      </c>
+      <c r="C18" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="D18" s="14" t="n">
+        <v>209</v>
+      </c>
+      <c r="E18" s="14" t="n">
+        <v>145</v>
+      </c>
+      <c r="F18" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H18" s="14" t="n">
+        <v>44</v>
+      </c>
+      <c r="I18" s="18" t="n">
         <f aca="false">IF(SUM(B18:F18,H18)=0,"",SUM(B18:F18,H18))</f>
-        <v/>
-      </c>
-      <c r="J18" s="18" t="str">
+        <v>1203</v>
+      </c>
+      <c r="J18" s="18" t="n">
         <f aca="false">IF(I18="","",1440-I18)</f>
-        <v/>
-      </c>
-      <c r="K18" s="16"/>
-      <c r="L18" s="16"/>
-      <c r="M18" s="16"/>
-      <c r="N18" s="17"/>
+        <v>237</v>
+      </c>
+      <c r="K18" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="L18" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="M18" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N18" s="17" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="14"/>
-      <c r="I19" s="18" t="str">
+      <c r="A19" s="13" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B19" s="14" t="n">
+        <v>377</v>
+      </c>
+      <c r="C19" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="D19" s="14" t="n">
+        <v>204</v>
+      </c>
+      <c r="E19" s="14" t="n">
+        <v>107</v>
+      </c>
+      <c r="F19" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="G19" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="14" t="n">
+        <v>88</v>
+      </c>
+      <c r="I19" s="18" t="n">
         <f aca="false">IF(SUM(B19:F19,H19)=0,"",SUM(B19:F19,H19))</f>
-        <v/>
-      </c>
-      <c r="J19" s="18" t="str">
+        <v>916</v>
+      </c>
+      <c r="J19" s="18" t="n">
         <f aca="false">IF(I19="","",1440-I19)</f>
-        <v/>
-      </c>
-      <c r="K19" s="16"/>
-      <c r="L19" s="16"/>
-      <c r="M19" s="16"/>
-      <c r="N19" s="17"/>
+        <v>524</v>
+      </c>
+      <c r="K19" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L19" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="M19" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N19" s="17" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="18" t="str">
+      <c r="A20" s="13" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B20" s="14" t="n">
+        <v>340</v>
+      </c>
+      <c r="C20" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="14" t="n">
+        <v>93</v>
+      </c>
+      <c r="E20" s="14" t="n">
+        <v>165</v>
+      </c>
+      <c r="F20" s="14" t="n">
+        <v>400</v>
+      </c>
+      <c r="G20" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="I20" s="18" t="n">
         <f aca="false">IF(SUM(B20:F20,H20)=0,"",SUM(B20:F20,H20))</f>
-        <v/>
-      </c>
-      <c r="J20" s="18" t="str">
+        <v>1013</v>
+      </c>
+      <c r="J20" s="18" t="n">
         <f aca="false">IF(I20="","",1440-I20)</f>
-        <v/>
-      </c>
-      <c r="K20" s="16"/>
-      <c r="L20" s="16"/>
-      <c r="M20" s="16"/>
-      <c r="N20" s="17"/>
+        <v>427</v>
+      </c>
+      <c r="K20" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L20" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="M20" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N20" s="17" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="13"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="18" t="str">
+      <c r="A21" s="13" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B21" s="14" t="n">
+        <v>448</v>
+      </c>
+      <c r="C21" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="D21" s="14" t="n">
+        <v>202</v>
+      </c>
+      <c r="E21" s="14" t="n">
+        <v>181</v>
+      </c>
+      <c r="F21" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="G21" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H21" s="14" t="n">
+        <v>49</v>
+      </c>
+      <c r="I21" s="18" t="n">
         <f aca="false">IF(SUM(B21:F21,H21)=0,"",SUM(B21:F21,H21))</f>
-        <v/>
-      </c>
-      <c r="J21" s="18" t="str">
+        <v>1040</v>
+      </c>
+      <c r="J21" s="18" t="n">
         <f aca="false">IF(I21="","",1440-I21)</f>
-        <v/>
-      </c>
-      <c r="K21" s="16"/>
-      <c r="L21" s="16"/>
-      <c r="M21" s="16"/>
-      <c r="N21" s="17"/>
+        <v>400</v>
+      </c>
+      <c r="K21" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="L21" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="M21" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="N21" s="17" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="13"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="14"/>
-      <c r="G22" s="14"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="18" t="str">
+      <c r="A22" s="13" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B22" s="14" t="n">
+        <v>351</v>
+      </c>
+      <c r="C22" s="14" t="n">
+        <v>45</v>
+      </c>
+      <c r="D22" s="14" t="n">
+        <v>161</v>
+      </c>
+      <c r="E22" s="14" t="n">
+        <v>134</v>
+      </c>
+      <c r="F22" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="G22" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" s="14" t="n">
+        <v>110</v>
+      </c>
+      <c r="I22" s="18" t="n">
         <f aca="false">IF(SUM(B22:F22,H22)=0,"",SUM(B22:F22,H22))</f>
-        <v/>
-      </c>
-      <c r="J22" s="18" t="str">
+        <v>1101</v>
+      </c>
+      <c r="J22" s="18" t="n">
         <f aca="false">IF(I22="","",1440-I22)</f>
-        <v/>
-      </c>
-      <c r="K22" s="16"/>
-      <c r="L22" s="16"/>
-      <c r="M22" s="16"/>
-      <c r="N22" s="17"/>
+        <v>339</v>
+      </c>
+      <c r="K22" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="L22" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="M22" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="N22" s="17" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="13"/>

</xml_diff>

<commit_message>
Updated till 12th September
</commit_message>
<xml_diff>
--- a/12625732.xlsx
+++ b/12625732.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="78">
   <si>
     <t xml:space="preserve">My Data, My Code</t>
   </si>
@@ -252,6 +252,9 @@
   </si>
   <si>
     <t xml:space="preserve">long lecture 10:20am-5pm, exhausted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">busy day</t>
   </si>
 </sst>
 </file>
@@ -1898,180 +1901,372 @@
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="13"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="18" t="str">
+      <c r="A23" s="13" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B23" s="14" t="n">
+        <v>381</v>
+      </c>
+      <c r="C23" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="D23" s="14" t="n">
+        <v>173</v>
+      </c>
+      <c r="E23" s="14" t="n">
+        <v>192</v>
+      </c>
+      <c r="F23" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="14" t="n">
+        <v>96</v>
+      </c>
+      <c r="I23" s="18" t="n">
         <f aca="false">IF(SUM(B23:F23,H23)=0,"",SUM(B23:F23,H23))</f>
-        <v/>
-      </c>
-      <c r="J23" s="18" t="str">
+        <v>902</v>
+      </c>
+      <c r="J23" s="18" t="n">
         <f aca="false">IF(I23="","",1440-I23)</f>
-        <v/>
-      </c>
-      <c r="K23" s="16"/>
-      <c r="L23" s="16"/>
-      <c r="M23" s="16"/>
-      <c r="N23" s="17"/>
+        <v>538</v>
+      </c>
+      <c r="K23" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L23" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M23" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N23" s="17" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="13"/>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="18" t="str">
+      <c r="A24" s="13" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B24" s="14" t="n">
+        <v>463</v>
+      </c>
+      <c r="C24" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="D24" s="14" t="n">
+        <v>143</v>
+      </c>
+      <c r="E24" s="14" t="n">
+        <v>159</v>
+      </c>
+      <c r="F24" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="14" t="n">
+        <v>127</v>
+      </c>
+      <c r="I24" s="18" t="n">
         <f aca="false">IF(SUM(B24:F24,H24)=0,"",SUM(B24:F24,H24))</f>
-        <v/>
-      </c>
-      <c r="J24" s="18" t="str">
+        <v>967</v>
+      </c>
+      <c r="J24" s="18" t="n">
         <f aca="false">IF(I24="","",1440-I24)</f>
-        <v/>
-      </c>
-      <c r="K24" s="16"/>
-      <c r="L24" s="16"/>
-      <c r="M24" s="16"/>
-      <c r="N24" s="17"/>
+        <v>473</v>
+      </c>
+      <c r="K24" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="L24" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M24" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="N24" s="17" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="13"/>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
-      <c r="G25" s="14"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="18" t="str">
+      <c r="A25" s="13" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B25" s="14" t="n">
+        <v>424</v>
+      </c>
+      <c r="C25" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="D25" s="14" t="n">
+        <v>199</v>
+      </c>
+      <c r="E25" s="14" t="n">
+        <v>47</v>
+      </c>
+      <c r="F25" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="G25" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H25" s="14" t="n">
+        <v>49</v>
+      </c>
+      <c r="I25" s="18" t="n">
         <f aca="false">IF(SUM(B25:F25,H25)=0,"",SUM(B25:F25,H25))</f>
-        <v/>
-      </c>
-      <c r="J25" s="18" t="str">
+        <v>899</v>
+      </c>
+      <c r="J25" s="18" t="n">
         <f aca="false">IF(I25="","",1440-I25)</f>
-        <v/>
-      </c>
-      <c r="K25" s="16"/>
-      <c r="L25" s="16"/>
-      <c r="M25" s="16"/>
-      <c r="N25" s="17"/>
+        <v>541</v>
+      </c>
+      <c r="K25" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L25" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="M25" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N25" s="17" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="13"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="14"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="18" t="str">
+      <c r="A26" s="13" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B26" s="14" t="n">
+        <v>434</v>
+      </c>
+      <c r="C26" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="D26" s="14" t="n">
+        <v>203</v>
+      </c>
+      <c r="E26" s="14" t="n">
+        <v>38</v>
+      </c>
+      <c r="F26" s="14" t="n">
+        <v>150</v>
+      </c>
+      <c r="G26" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H26" s="14" t="n">
+        <v>83</v>
+      </c>
+      <c r="I26" s="18" t="n">
         <f aca="false">IF(SUM(B26:F26,H26)=0,"",SUM(B26:F26,H26))</f>
-        <v/>
-      </c>
-      <c r="J26" s="18" t="str">
+        <v>968</v>
+      </c>
+      <c r="J26" s="18" t="n">
         <f aca="false">IF(I26="","",1440-I26)</f>
-        <v/>
-      </c>
-      <c r="K26" s="16"/>
-      <c r="L26" s="16"/>
-      <c r="M26" s="16"/>
-      <c r="N26" s="17"/>
+        <v>472</v>
+      </c>
+      <c r="K26" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L26" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="M26" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="N26" s="17" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="13"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="18" t="str">
+      <c r="A27" s="13" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B27" s="14" t="n">
+        <v>340</v>
+      </c>
+      <c r="C27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="14" t="n">
+        <v>65</v>
+      </c>
+      <c r="E27" s="14" t="n">
+        <v>27</v>
+      </c>
+      <c r="F27" s="14" t="n">
+        <v>400</v>
+      </c>
+      <c r="G27" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="I27" s="18" t="n">
         <f aca="false">IF(SUM(B27:F27,H27)=0,"",SUM(B27:F27,H27))</f>
-        <v/>
-      </c>
-      <c r="J27" s="18" t="str">
+        <v>847</v>
+      </c>
+      <c r="J27" s="18" t="n">
         <f aca="false">IF(I27="","",1440-I27)</f>
-        <v/>
-      </c>
-      <c r="K27" s="16"/>
-      <c r="L27" s="16"/>
-      <c r="M27" s="16"/>
-      <c r="N27" s="17"/>
+        <v>593</v>
+      </c>
+      <c r="K27" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L27" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="M27" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N27" s="17" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="13"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="18" t="str">
+      <c r="A28" s="13" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B28" s="14" t="n">
+        <v>335</v>
+      </c>
+      <c r="C28" s="14" t="n">
+        <v>45</v>
+      </c>
+      <c r="D28" s="14" t="n">
+        <v>131</v>
+      </c>
+      <c r="E28" s="14" t="n">
+        <v>171</v>
+      </c>
+      <c r="F28" s="14" t="n">
+        <v>150</v>
+      </c>
+      <c r="G28" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H28" s="14" t="n">
+        <v>82</v>
+      </c>
+      <c r="I28" s="18" t="n">
         <f aca="false">IF(SUM(B28:F28,H28)=0,"",SUM(B28:F28,H28))</f>
-        <v/>
-      </c>
-      <c r="J28" s="18" t="str">
+        <v>914</v>
+      </c>
+      <c r="J28" s="18" t="n">
         <f aca="false">IF(I28="","",1440-I28)</f>
-        <v/>
-      </c>
-      <c r="K28" s="16"/>
-      <c r="L28" s="16"/>
-      <c r="M28" s="16"/>
-      <c r="N28" s="17"/>
+        <v>526</v>
+      </c>
+      <c r="K28" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="L28" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M28" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N28" s="17" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="13"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="18" t="str">
+      <c r="A29" s="13" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B29" s="14" t="n">
+        <v>450</v>
+      </c>
+      <c r="C29" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="D29" s="14" t="n">
+        <v>109</v>
+      </c>
+      <c r="E29" s="14" t="n">
+        <v>229</v>
+      </c>
+      <c r="F29" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="G29" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H29" s="14" t="n">
+        <v>106</v>
+      </c>
+      <c r="I29" s="18" t="n">
         <f aca="false">IF(SUM(B29:F29,H29)=0,"",SUM(B29:F29,H29))</f>
-        <v/>
-      </c>
-      <c r="J29" s="18" t="str">
+        <v>1044</v>
+      </c>
+      <c r="J29" s="18" t="n">
         <f aca="false">IF(I29="","",1440-I29)</f>
-        <v/>
-      </c>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16"/>
-      <c r="M29" s="16"/>
-      <c r="N29" s="17"/>
+        <v>396</v>
+      </c>
+      <c r="K29" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L29" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M29" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="N29" s="17" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="13"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="18" t="str">
+      <c r="A30" s="13" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B30" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C30" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="D30" s="14" t="n">
+        <v>169</v>
+      </c>
+      <c r="E30" s="14" t="n">
+        <v>81</v>
+      </c>
+      <c r="F30" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="14" t="n">
+        <v>103</v>
+      </c>
+      <c r="I30" s="18" t="n">
         <f aca="false">IF(SUM(B30:F30,H30)=0,"",SUM(B30:F30,H30))</f>
-        <v/>
-      </c>
-      <c r="J30" s="18" t="str">
+        <v>848</v>
+      </c>
+      <c r="J30" s="18" t="n">
         <f aca="false">IF(I30="","",1440-I30)</f>
-        <v/>
-      </c>
-      <c r="K30" s="16"/>
-      <c r="L30" s="16"/>
-      <c r="M30" s="16"/>
-      <c r="N30" s="17"/>
+        <v>592</v>
+      </c>
+      <c r="K30" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="L30" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="M30" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N30" s="17" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="13"/>

</xml_diff>